<commit_message>
version con falla en horarios
</commit_message>
<xml_diff>
--- a/sistema de registro de docentes/Resources/materias.xlsx
+++ b/sistema de registro de docentes/Resources/materias.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\PROYECTO\proyecto registro de asistencia profesores\sistema de registro de docentes\sistema de registro de docentes\Resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96A740DC-16F7-433F-A4F6-334021397F27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5882E475-1CDC-4E2A-A46A-887B1917169E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ING. DE SISTEMAS" sheetId="5" r:id="rId1"/>
     <sheet name="ING. MECATRONICA" sheetId="7" r:id="rId2"/>
-    <sheet name="ING. EN TELECOMUNICACIONES" sheetId="8" r:id="rId3"/>
-    <sheet name="ING. DE SIS. ELECTRONICOS" sheetId="6" r:id="rId4"/>
+    <sheet name="ING. DE TELECOMUNICACIONES" sheetId="8" r:id="rId3"/>
+    <sheet name="ING. DE SISTEMAS ELECTRONICOS" sheetId="6" r:id="rId4"/>
   </sheets>
   <calcPr calcId="162913"/>
 </workbook>

</xml_diff>